<commit_message>
Auto-archive: Daily PIB UPSC Brief 2026-10-22
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-21.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-21.xlsx
@@ -42,7 +42,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
         <bgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -100,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -120,7 +126,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -489,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -555,7 +564,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>DARE/ICAR Undertakes Nearly 4,000 Cleanliness Drives under Swachhata Special Campaign 6.0</t>
+          <t>“Solar panels above, thriving crops below”: Union Minister Shri Shivraj Singh Chouhan inaugurates the 7th AgriVoltaics World Conference at Bharat Mandapam</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -570,7 +579,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325852</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326152</t>
         </is>
       </c>
     </row>
@@ -585,27 +594,28 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Defence</t>
+          <t>Ministry of Agriculture &amp;
+Farmers Welfare</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>MOD INKS ₹ 770 Cr CONTRACT TO PROCURE IMPROVED LOW LEVEL LIGHT WEIGHT RADARS FOR INDIAN ARMY</t>
+          <t>Ministry of Agriculture &amp; Farmers Welfare to Launch ‘Khet Bachao Abhiyan – Rabi 2026’ tomorrow; Campaign to Continue Till 30 November</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>indian army</t>
+          <t>agriculture</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: indian army</t>
+          <t>Aligned with General Studies 3 topics: agriculture</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325933</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326112</t>
         </is>
       </c>
     </row>
@@ -613,34 +623,35 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Law and Justice</t>
+          <t>Ministry of Agriculture &amp;
+Farmers Welfare</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Law Commission of India to organise National Conference on ‘Co-operative Federalism and Law Reforms: National and State Perspectives’</t>
+          <t>DARE/ICAR Undertakes Nearly 4,000 Cleanliness Drives under Swachhata Special Campaign 6.0</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>law commission</t>
+          <t>agriculture</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: law commission</t>
+          <t>Aligned with General Studies 3 topics: agriculture</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325856</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325852</t>
         </is>
       </c>
     </row>
@@ -648,32 +659,452 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Culture</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Hon’ble President of India Smt. Droupadi Murmu presents 65th National Exhibition of Art and 3rd Print Biennale India awards to artists, celebrating India’s rich artistic heritage and contemporary creativity</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>heritage</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 1 topics: heritage</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326116</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>GS-3</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>33rd EDITION OF SINGAPORE-INDIA MARITIME BILATERAL EXERCISE (SIMBEX-2026) COMMENCES AT VISAKHAPATNAM</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>bilateral exercise</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: bilateral exercise</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326348</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>INDIAN AIR FORCE ENGAGES INDUSTRY OUTREACH PROGRAMME ON UNMANNED AND AUTONOMOUS SYSTEMS ROADMAP ON 21 OCT 26</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>indian air force</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: indian air force</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326184</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>CONCLUSION OF THE NINTH EDITION OF INDIA-BRAZIL-SOUTH AFRICA MARITIME EXERCISE (IBSAMAR IX 2026)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Internal &amp; External Security</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Strategic policy update from nodal ministry (Ministry of Defence): Internal &amp; External Security / Defence Capabilities</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326117</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>MOD INKS ₹ 770 Cr CONTRACT TO PROCURE IMPROVED LOW LEVEL LIGHT WEIGHT RADARS FOR INDIAN ARMY</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>indian army</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: indian army</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325933</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>CAQM holds meeting with Delhi Government agencies to review Dust Pollution issues and strengthen Air Pollution Mitigation</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>climate change, caqm</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326148</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>CAQM invokes Stage-I of GRAP in Delhi-NCR with immediate effect amid sharp rise in AQI</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>climate change, caqm</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326133</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Finance</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>India and New Zealand sign Memorandum of Cooperation (MoC) on Electronic Origin Data Exchange to Facilitate Bilateral Trade Under the India-New Zealand Free Trade Agreement (FTA)</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Economic Governance &amp; Fiscal Policy</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Strategic policy update from nodal ministry (Ministry of Finance): Economic Governance &amp; Fiscal Policy</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326043</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Law Commission of India to organise National Conference on ‘Co-operative Federalism and Law Reforms: National and State Perspectives’</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>law commission</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: law commission</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325856</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Micro,Small &amp; Medium Enterprises</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>National Institute for Micro, Small and Medium Enterprises (ni-msme) strengthens MSMEs through Capacity Building, Entrepreneurship Development and Digital Empowerment</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>msme</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: msme</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326147</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of New and Renewable Energy</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>India hosts Agrivoltaics World Conference 2026</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>renewable energy</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: renewable energy</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326072</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of New and Renewable Energy</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>India hosts Agrivoltaics World Conference 2026 for the first time in the Global South</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>renewable energy</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: renewable energy</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326059</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Armed Forces Headquarters Association (AFHQ) appreciates timely promotions under PM Narendra Modi’s Leadership; Discusses employee issues with Dr Jitendra Singh</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>armed forces</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Aligned with General Studies 3 topics: armed forces</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325959</t>
         </is>
@@ -685,6 +1116,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -696,7 +1139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -708,32 +1151,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>S.No.</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Classification</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Paper</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Ministry</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Headline</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>PIB URL</t>
         </is>
@@ -760,12 +1203,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PRESIDENT OF INDIA PRESENTS LALIT KALA AKADEMI AWARDS TO SELECTED ARTISTS OF THE 65TH NATIONAL EXHIBITION OF ART</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325915</t>
+          <t>PRESIDENT OF INDIA TO VISIT CHHATTISGARH FROM OCTOBER 22 TO 23</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326091</t>
         </is>
       </c>
     </row>
@@ -780,22 +1223,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Routine/Ceremonial</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>President's Secretariat</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Prime Minister condoles the passing of Thiru Vummidi Ethiraj Ji</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325908</t>
+          <t>PRESIDENT OF INDIA PRESENTS LALIT KALA AKADEMI AWARDS TO SELECTED ARTISTS OF THE 65TH NATIONAL EXHIBITION OF ART</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325915</t>
         </is>
       </c>
     </row>
@@ -820,12 +1263,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Prime Minister shares an article by Union Minister Shri Shivraj Singh Chouhan highlighting the role of technology and research in transforming agriculture and improving farmers' lives</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325772</t>
+          <t>Prime Minister congratulates Shailesh Kumar on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326319</t>
         </is>
       </c>
     </row>
@@ -850,12 +1293,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Prime Minister shares an article by Union Ministers Shri Pralhad Joshi and Shri Shivraj Singh Chouhan highlighting the potential of agrivoltaics to boost farmers' incomes and advance rural prosperity</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325735</t>
+          <t>Prime Minister congratulates Ravi Kartik Budigina on winning Silver at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326265</t>
         </is>
       </c>
     </row>
@@ -880,12 +1323,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Prime Minister pays tributes to brave police personnel on Police Commemoration Day</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325655</t>
+          <t>Prime Minister congratulates Himanshu Nandal on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326263</t>
         </is>
       </c>
     </row>
@@ -910,12 +1353,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Prime Minister shares a Sanskrit Subhashitam, highlighting the enduring gratitude and benevolence of noble individuals</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325652</t>
+          <t>Prime Minister congratulates Pranav Desai on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326258</t>
         </is>
       </c>
     </row>
@@ -925,28 +1368,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture &amp;
-Farmers Welfare</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>DARE/ICAR Undertakes Nearly 4,000 Cleanliness Drives under Swachhata Special Campaign 6.0</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325852</t>
+          <t>Prime Minister congratulates Rohit Kumar on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326256</t>
         </is>
       </c>
     </row>
@@ -961,22 +1403,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ministry of Coal</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CCO's SUVIKALP Initiative Advances Sustainable Mine Repurposing, Receives SKOCH Gold Award 2026</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325820</t>
+          <t>Prime Minister congratulates Simran on winning Gold at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326163</t>
         </is>
       </c>
     </row>
@@ -991,22 +1433,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ministry of Defence</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Department of Military Affairs Reviews Over 2.46 Lakh Files During Special Campaign 6</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326033</t>
+          <t>Prime Minister congratulates Karamjyoti on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326161</t>
         </is>
       </c>
     </row>
@@ -1016,27 +1458,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ministry of Defence</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MOD INKS ₹ 770 Cr CONTRACT TO PROCURE IMPROVED LOW LEVEL LIGHT WEIGHT RADARS FOR INDIAN ARMY</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325933</t>
+          <t>Prime Minister congratulates Sukhchain on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326142</t>
         </is>
       </c>
     </row>
@@ -1051,22 +1493,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Ministry of Defence</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ARMY COMMANDERS’ CONFERENCE COMMENCES TODAY</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325911</t>
+          <t>Prime Minister congratulates Mohammad Basil M on winning Silver at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326140</t>
         </is>
       </c>
     </row>
@@ -1086,17 +1528,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ministry of Home Affairs</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Union Home Minister and Minister of Cooperation Shri Amit Shah pays tribute to police personnel who laid down their lives in line of duty at National Police Memorial on the occasion of Police Commemoration Day and addresses the ceremony</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325853</t>
+          <t>Prime Minister congratulates Dilip Gavit on winning Gold at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326138</t>
         </is>
       </c>
     </row>
@@ -1106,27 +1548,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Ministry of Law and Justice</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Law Commission of India to organise National Conference on ‘Co-operative Federalism and Law Reforms: National and State Perspectives’</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325856</t>
+          <t>Prime Minister congratulates Ravi Rongali on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326126</t>
         </is>
       </c>
     </row>
@@ -1141,22 +1583,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Union Minister joins Dr Jitendra Singh joins an e-waste disposal activity at DoPT under Special Campaign 6.0</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325966</t>
+          <t>Prime Minister congratulates Preeti Pal on winning Silver at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326123</t>
         </is>
       </c>
     </row>
@@ -1166,27 +1608,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Armed Forces Headquarters Association (AFHQ) appreciates timely promotions under PM Narendra Modi’s Leadership; Discusses employee issues with Dr Jitendra Singh</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325959</t>
+          <t>Prime Minister congratulates Kasthuri Rajamani on winning Silver at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326119</t>
         </is>
       </c>
     </row>
@@ -1201,22 +1643,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Ministry of Science &amp; Technology</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pulsing signals reveal hidden structure around a famous neutron star</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326032</t>
+          <t>Prime Minister congratulates Manjeet on winning Silver at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326113</t>
         </is>
       </c>
     </row>
@@ -1231,22 +1673,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Ministry of Social Justice &amp; Empowerment</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>From Financial Hardship to Academic Aspirations</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326007</t>
+          <t>Prime Minister congratulates Bhagyashree Jadhav on winning Silver at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326111</t>
         </is>
       </c>
     </row>
@@ -1261,22 +1703,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Ministry of Social Justice &amp; Empowerment</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>A New Beginning Built on Equality</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325991</t>
+          <t>Prime Minister congratulates Parveen on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326105</t>
         </is>
       </c>
     </row>
@@ -1291,22 +1733,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>UPSC</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Union Public Service Commission announces Recruitment Results for the month of September, 2026</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325768</t>
+          <t>Prime Minister congratulates Mohd Yasser on winning Silver at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326103</t>
         </is>
       </c>
     </row>
@@ -1321,22 +1763,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>PIB Backgrounder</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Transforming Wastewater Treatment</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325989</t>
+          <t>Prime Minister congratulates Sachin Khilari on winning Gold at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326102</t>
         </is>
       </c>
     </row>
@@ -1351,22 +1793,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PIB Backgrounder</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SARAS Mela 2026</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325711</t>
+          <t>Prime Minister congratulates Rakeshbhai Bhatt on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326101</t>
         </is>
       </c>
     </row>
@@ -1381,20 +1823,1433 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Prime Minister congratulates Banti on winning Silver at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326100</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Prime Minister congratulates Praveen Kumar on winning Gold at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326098</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Prime Minister congratulates Ayush Verma on winning Gold at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326097</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Prime Minister congratulates Sheetal Devi and Payal Nag on winning Silver at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326095</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Prime Minister congratulates Anubhav Choudhary on winning Bronze at the Asian Para Games</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326093</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Prime Minister condoles the passing of Thiru Vummidi Ethiraj Ji</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325908</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Prime Minister shares an article by Union Minister Shri Shivraj Singh Chouhan highlighting the role of technology and research in transforming agriculture and improving farmers' lives</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325772</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Prime Minister shares an article by Union Ministers Shri Pralhad Joshi and Shri Shivraj Singh Chouhan highlighting the potential of agrivoltaics to boost farmers' incomes and advance rural prosperity</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325735</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Prime Minister pays tributes to brave police personnel on Police Commemoration Day</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325655</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Prime Minister's Office</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Prime Minister shares a Sanskrit Subhashitam, highlighting the enduring gratitude and benevolence of noble individuals</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325652</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Ministry of Agriculture &amp;
+Farmers Welfare</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>“Solar panels above, thriving crops below”: Union Minister Shri Shivraj Singh Chouhan inaugurates the 7th AgriVoltaics World Conference at Bharat Mandapam</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326152</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Ministry of Agriculture &amp;
+Farmers Welfare</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Ministry of Agriculture &amp; Farmers Welfare to Launch ‘Khet Bachao Abhiyan – Rabi 2026’ tomorrow; Campaign to Continue Till 30 November</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326112</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Ministry of Agriculture &amp;
+Farmers Welfare</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>DARE/ICAR Undertakes Nearly 4,000 Cleanliness Drives under Swachhata Special Campaign 6.0</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325852</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>General/Administrative</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Ministry of Coal</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>CCO's SUVIKALP Initiative Advances Sustainable Mine Repurposing, Receives SKOCH Gold Award 2026</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325820</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Ministry of Commerce &amp; Industry</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Union Minister of Commerce and Industry Shri Piyush Goyal to Visit Germany and the Netherlands to Strengthen Trade, Investment and Industrial Cooperation</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326057</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Ministry of Commerce &amp; Industry</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PROVISIONAL INDEX OF CORE INDUSTRIES FOR THE MONTH OF SEPTEMBER 2026, AND FINAL INDEX FOR THE MONTH OF AUGUST 2026 WITH BASE YEAR 2022-23</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326038</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Ministry of Culture</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Hon’ble President of India Smt. Droupadi Murmu presents 65th National Exhibition of Art and 3rd Print Biennale India awards to artists, celebrating India’s rich artistic heritage and contemporary creativity</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326116</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>33rd EDITION OF SINGAPORE-INDIA MARITIME BILATERAL EXERCISE (SIMBEX-2026) COMMENCES AT VISAKHAPATNAM</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326348</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>INDIAN AIR FORCE ENGAGES INDUSTRY OUTREACH PROGRAMME ON UNMANNED AND AUTONOMOUS SYSTEMS ROADMAP ON 21 OCT 26</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326184</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>CONCLUSION OF THE NINTH EDITION OF INDIA-BRAZIL-SOUTH AFRICA MARITIME EXERCISE (IBSAMAR IX 2026)</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326117</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Department of Military Affairs Reviews Over 2.46 Lakh Files During Special Campaign 6</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326033</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>MOD INKS ₹ 770 Cr CONTRACT TO PROCURE IMPROVED LOW LEVEL LIGHT WEIGHT RADARS FOR INDIAN ARMY</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325933</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ARMY COMMANDERS’ CONFERENCE COMMENCES TODAY</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325911</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>CAQM holds meeting with Delhi Government agencies to review Dust Pollution issues and strengthen Air Pollution Mitigation</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326148</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CAQM invokes Stage-I of GRAP in Delhi-NCR with immediate effect amid sharp rise in AQI</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326133</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Ministry of Finance</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>DRI seizes more than 9 kg methamphetamine in intensified crackdown on synthetic drug trafficking in Bhopal; One held</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326107</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Ministry of Finance</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>India and New Zealand sign Memorandum of Cooperation (MoC) on Electronic Origin Data Exchange to Facilitate Bilateral Trade Under the India-New Zealand Free Trade Agreement (FTA)</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326043</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Ministry of Home Affairs</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Union Home Secretary Shri Govind Mohan addresses Press Conference in New Delhi on Rashtriya Ekta Diwas 2026 and Bharat Parv 2026 celebrations to be held at Ekta Nagar, Gujarat</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326165</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Routine/Ceremonial</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Ministry of Home Affairs</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Union Home Minister and Minister of Cooperation Shri Amit Shah pays tribute to police personnel who laid down their lives in line of duty at National Police Memorial on the occasion of Police Commemoration Day and addresses the ceremony</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325853</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Ministry of Information &amp; Broadcasting</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>NFDC–NFAI to present a Four-Day Ritwik Ghatak Film Festival in Pune, offering a rare glimpse into the Filmmaker’s Diverse Cinematic Legacy</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326081</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Law Commission of India to organise National Conference on ‘Co-operative Federalism and Law Reforms: National and State Perspectives’</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325856</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Ministry of Micro,Small &amp; Medium Enterprises</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>National Institute for Micro, Small and Medium Enterprises (ni-msme) strengthens MSMEs through Capacity Building, Entrepreneurship Development and Digital Empowerment</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326147</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Ministry of New and Renewable Energy</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>India hosts Agrivoltaics World Conference 2026</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326072</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Ministry of New and Renewable Energy</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>India hosts Agrivoltaics World Conference 2026 for the first time in the Global South</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326059</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Union Minister joins Dr Jitendra Singh joins an e-waste disposal activity at DoPT under Special Campaign 6.0</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325966</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Ministry of Personnel, Public Grievances &amp; Pensions</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Armed Forces Headquarters Association (AFHQ) appreciates timely promotions under PM Narendra Modi’s Leadership; Discusses employee issues with Dr Jitendra Singh</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325959</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Ministry of Science &amp; Technology</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Pulsing signals reveal hidden structure around a famous neutron star</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326032</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>National Action Plan For Drug Demand Reduction (NAPDDR)</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326124</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>8 Days Shilp Samagam Mela 2026 Begins in Guwahati Today</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326056</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>From Financial Hardship to Academic Aspirations</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326007</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>A New Beginning Built on Equality</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325991</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Ministry of Textiles</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Deep Cleaning Exercise under Special Campaign 6.0</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326129</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Ministry of Women and Child Development</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Ministry of Women and Child Development to Organize Dedicated Nationwide Drive on 30th October Under Special Campaign 6</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326141</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Ministry of Youth Affairs and Sports</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Union MoS Raksha Khadse, Guest of Honour at Chhattisgarh Hockey League Opening Ceremony, Calls It a Major Step Towards Strengthening Grassroots Hockey</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2326255</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>UPSC</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Union Public Service Commission announces Recruitment Results for the month of September, 2026</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325768</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>PIB Backgrounder</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Transforming Wastewater Treatment</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325989</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>PIB Backgrounder</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>SARAS Mela 2026</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325711</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
         <is>
           <t>Ministry of Chemicals and Fertilizers - Department of Chemicals and Petrochemicals</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>14th India Chem 2026 to Bring Global Chemicals and Petrochemicals Industry Together in Mumbai from October 22</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F70" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2325901</t>
         </is>
@@ -1424,6 +3279,53 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>